<commit_message>
Added Per Y Feature Selection
</commit_message>
<xml_diff>
--- a/Test_Results.xlsx
+++ b/Test_Results.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="49">
   <si>
     <t>Data Selected</t>
   </si>
@@ -79,12 +79,6 @@
   </si>
   <si>
     <t>CGC_5TH_STG_DISCH_PRES</t>
-  </si>
-  <si>
-    <t>R² = 0.9097</t>
-  </si>
-  <si>
-    <t>R² = 0.6410</t>
   </si>
   <si>
     <t>CGC Power</t>
@@ -306,12 +300,24 @@
   <si>
     <t>DMCTF feed</t>
   </si>
+  <si>
+    <t>KT1301 TURBINE SPEED (RPM)</t>
+  </si>
+  <si>
+    <t>Combined Feature Selection</t>
+  </si>
+  <si>
+    <t>Individual Feature Selection</t>
+  </si>
+  <si>
+    <t>CGC_3RD_STG_SUCT_PRESS</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -394,13 +400,31 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="5" tint="0.39997558519241921"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -416,16 +440,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -457,6 +476,39 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -493,13 +545,13 @@
         <xdr:from>
           <xdr:col>3</xdr:col>
           <xdr:colOff>0</xdr:colOff>
-          <xdr:row>83</xdr:row>
+          <xdr:row>90</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>3</xdr:col>
           <xdr:colOff>914400</xdr:colOff>
-          <xdr:row>84</xdr:row>
+          <xdr:row>91</xdr:row>
           <xdr:rowOff>44450</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
@@ -540,13 +592,13 @@
         <xdr:from>
           <xdr:col>3</xdr:col>
           <xdr:colOff>0</xdr:colOff>
-          <xdr:row>93</xdr:row>
+          <xdr:row>100</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>3</xdr:col>
           <xdr:colOff>914400</xdr:colOff>
-          <xdr:row>94</xdr:row>
+          <xdr:row>101</xdr:row>
           <xdr:rowOff>44450</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
@@ -848,7 +900,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:G101"/>
+  <dimension ref="A1:J108"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="11.36328125" customWidth="1"/>
@@ -858,9 +910,10 @@
     <col min="5" max="5" width="20.26953125" customWidth="1"/>
     <col min="6" max="6" width="26.26953125" customWidth="1"/>
     <col min="7" max="7" width="20.36328125" customWidth="1"/>
+    <col min="10" max="10" width="20.08984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:10">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -883,446 +936,663 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="18">
-      <c r="A2">
+    <row r="2" spans="1:10" ht="18">
+      <c r="A2" s="16">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="17">
+        <v>0.90900000000000003</v>
+      </c>
+      <c r="F2" s="18" t="s">
+        <v>8</v>
+      </c>
+      <c r="G2" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="18">
+      <c r="A3" s="16"/>
+      <c r="B3" s="16"/>
+      <c r="C3" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="17">
+        <v>0.64100000000000001</v>
+      </c>
+      <c r="F3" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="G3" s="16"/>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4" s="16"/>
+      <c r="B4" s="16"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="16"/>
+      <c r="F4" s="18" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4" s="16"/>
+      <c r="I4" s="16"/>
+      <c r="J4" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="A5" s="16"/>
+      <c r="B5" s="16"/>
+      <c r="C5" s="16"/>
+      <c r="D5" s="16"/>
+      <c r="E5" s="16"/>
+      <c r="F5" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" s="16"/>
+      <c r="I5" s="13"/>
+      <c r="J5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="A6" s="16"/>
+      <c r="B6" s="16"/>
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" s="16"/>
+    </row>
+    <row r="7" spans="1:10">
+      <c r="A7" s="16"/>
+      <c r="B7" s="16"/>
+      <c r="C7" s="16"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="G7" s="16"/>
+    </row>
+    <row r="8" spans="1:10" s="24" customFormat="1">
+      <c r="F8" s="25"/>
+    </row>
+    <row r="9" spans="1:10">
+      <c r="A9" s="13">
+        <v>1</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D9" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="E9" s="13">
+        <v>0.83077177017733395</v>
+      </c>
+      <c r="F9" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="G9" s="13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10">
+      <c r="A10" s="13"/>
+      <c r="B10" s="13"/>
+      <c r="C10" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="D10" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="E10" s="13">
+        <v>0.58318588022978002</v>
+      </c>
+      <c r="F10" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="G10" s="13"/>
+    </row>
+    <row r="11" spans="1:10">
+      <c r="A11" s="13"/>
+      <c r="B11" s="13"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="E11" s="13"/>
+      <c r="F11" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="G11" s="13"/>
+    </row>
+    <row r="12" spans="1:10">
+      <c r="A12" s="13"/>
+      <c r="B12" s="13"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="E12" s="13"/>
+      <c r="F12" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="G12" s="13"/>
+    </row>
+    <row r="13" spans="1:10">
+      <c r="A13" s="13"/>
+      <c r="B13" s="13"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="E13" s="13"/>
+      <c r="F13" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="G13" s="13"/>
+    </row>
+    <row r="14" spans="1:10">
+      <c r="A14" s="13"/>
+      <c r="B14" s="13"/>
+      <c r="C14" s="13"/>
+      <c r="D14" s="13"/>
+      <c r="E14" s="13"/>
+      <c r="F14" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="G14" s="13"/>
+    </row>
+    <row r="16" spans="1:10">
+      <c r="A16" s="16">
+        <v>2</v>
+      </c>
+      <c r="B16" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="C16" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="D16" s="20" t="s">
+        <v>43</v>
+      </c>
+      <c r="E16" s="18">
+        <v>-1.05992909334717E-2</v>
+      </c>
+      <c r="F16" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G16" s="16" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="18">
-      <c r="C3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3" s="4" t="s">
+    <row r="17" spans="1:7">
+      <c r="A17" s="16"/>
+      <c r="B17" s="16"/>
+      <c r="C17" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="D17" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="E17" s="18">
+        <v>0.75641858263035999</v>
+      </c>
+      <c r="F17" s="18" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="C4" s="3"/>
-      <c r="D4" t="s">
-        <v>16</v>
-      </c>
-      <c r="F4" s="2" t="s">
+      <c r="G17" s="16"/>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18" s="16"/>
+      <c r="B18" s="16"/>
+      <c r="C18" s="16"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="16"/>
+      <c r="F18" s="18" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="F5" s="2" t="s">
+      <c r="G18" s="16"/>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19" s="16"/>
+      <c r="B19" s="16"/>
+      <c r="C19" s="16"/>
+      <c r="D19" s="21"/>
+      <c r="E19" s="16"/>
+      <c r="F19" s="18" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="F6" s="2" t="s">
+      <c r="G19" s="16"/>
+    </row>
+    <row r="20" spans="1:7">
+      <c r="A20" s="16"/>
+      <c r="B20" s="16"/>
+      <c r="C20" s="16"/>
+      <c r="D20" s="22"/>
+      <c r="E20" s="16"/>
+      <c r="F20" s="18" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="7" spans="1:7">
-      <c r="F7" s="2" t="s">
+      <c r="G20" s="16"/>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21" s="16"/>
+      <c r="B21" s="16"/>
+      <c r="C21" s="16"/>
+      <c r="D21" s="23"/>
+      <c r="E21" s="16"/>
+      <c r="F21" s="18" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="9" spans="1:7">
-      <c r="A9">
+      <c r="G21" s="16"/>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="D22" s="2"/>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23" s="13">
         <v>2</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B23" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D23" s="26" t="s">
+        <v>43</v>
+      </c>
+      <c r="E23" s="14">
+        <v>0.54235839056214397</v>
+      </c>
+      <c r="F23" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="G23" s="13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7">
+      <c r="A24" s="13"/>
+      <c r="B24" s="13"/>
+      <c r="C24" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="D24" s="26" t="s">
+        <v>45</v>
+      </c>
+      <c r="E24" s="14">
+        <v>0.865024831702778</v>
+      </c>
+      <c r="F24" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="G24" s="13"/>
+    </row>
+    <row r="25" spans="1:7">
+      <c r="A25" s="13"/>
+      <c r="B25" s="13"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="27"/>
+      <c r="E25" s="13"/>
+      <c r="F25" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="G25" s="13"/>
+    </row>
+    <row r="26" spans="1:7">
+      <c r="A26" s="13"/>
+      <c r="B26" s="13"/>
+      <c r="C26" s="13"/>
+      <c r="D26" s="27"/>
+      <c r="E26" s="13"/>
+      <c r="F26" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="G26" s="13"/>
+    </row>
+    <row r="27" spans="1:7">
+      <c r="A27" s="13"/>
+      <c r="B27" s="13"/>
+      <c r="C27" s="13"/>
+      <c r="D27" s="27"/>
+      <c r="E27" s="13"/>
+      <c r="F27" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="G27" s="13"/>
+    </row>
+    <row r="28" spans="1:7">
+      <c r="A28" s="13"/>
+      <c r="B28" s="13"/>
+      <c r="C28" s="13"/>
+      <c r="D28" s="27"/>
+      <c r="E28" s="13"/>
+      <c r="F28" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="G28" s="13"/>
+    </row>
+    <row r="29" spans="1:7">
+      <c r="D29" s="2"/>
+    </row>
+    <row r="30" spans="1:7">
+      <c r="D30" s="2"/>
+    </row>
+    <row r="31" spans="1:7">
+      <c r="D31" s="2"/>
+    </row>
+    <row r="32" spans="1:7">
+      <c r="D32" s="2"/>
+    </row>
+    <row r="33" spans="4:4">
+      <c r="D33" s="2"/>
+    </row>
+    <row r="34" spans="4:4">
+      <c r="D34" s="2"/>
+    </row>
+    <row r="35" spans="4:4">
+      <c r="D35" s="2"/>
+    </row>
+    <row r="36" spans="4:4">
+      <c r="D36" s="2"/>
+    </row>
+    <row r="37" spans="4:4">
+      <c r="D37" s="2"/>
+    </row>
+    <row r="38" spans="4:4">
+      <c r="D38" s="2"/>
+    </row>
+    <row r="39" spans="4:4">
+      <c r="D39" s="2"/>
+    </row>
+    <row r="40" spans="4:4">
+      <c r="D40" s="2"/>
+    </row>
+    <row r="41" spans="4:4">
+      <c r="D41" s="2"/>
+    </row>
+    <row r="42" spans="4:4">
+      <c r="D42" s="2"/>
+    </row>
+    <row r="43" spans="4:4">
+      <c r="D43" s="2"/>
+    </row>
+    <row r="44" spans="4:4">
+      <c r="D44" s="2"/>
+    </row>
+    <row r="45" spans="4:4">
+      <c r="D45" s="2"/>
+    </row>
+    <row r="46" spans="4:4">
+      <c r="D46" s="2"/>
+    </row>
+    <row r="47" spans="4:4">
+      <c r="D47" s="2"/>
+    </row>
+    <row r="48" spans="4:4">
+      <c r="D48" s="2"/>
+    </row>
+    <row r="49" spans="4:4">
+      <c r="D49" s="2"/>
+    </row>
+    <row r="50" spans="4:4">
+      <c r="D50" s="3"/>
+    </row>
+    <row r="51" spans="4:4">
+      <c r="D51" s="3"/>
+    </row>
+    <row r="53" spans="4:4">
+      <c r="D53" s="3"/>
+    </row>
+    <row r="54" spans="4:4">
+      <c r="D54" s="3"/>
+    </row>
+    <row r="55" spans="4:4">
+      <c r="D55" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="C9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D9" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="E9" s="2">
-        <v>-1.05992909334717E-2</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="G9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7">
-      <c r="C10" t="s">
+    </row>
+    <row r="56" spans="4:4">
+      <c r="D56" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="D10" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="E10" s="2">
-        <v>0.75641858263035999</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7">
-      <c r="F11" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7">
-      <c r="D12" s="7"/>
-      <c r="F12" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7">
-      <c r="D13" s="5"/>
-      <c r="F13" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7">
-      <c r="D14" s="5"/>
-      <c r="F14" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7">
-      <c r="D15" s="5"/>
-    </row>
-    <row r="16" spans="1:7">
-      <c r="D16" s="5"/>
-    </row>
-    <row r="17" spans="4:4">
-      <c r="D17" s="7"/>
-    </row>
-    <row r="18" spans="4:4">
-      <c r="D18" s="5"/>
-    </row>
-    <row r="19" spans="4:4">
-      <c r="D19" s="5"/>
-    </row>
-    <row r="20" spans="4:4">
-      <c r="D20" s="5"/>
-    </row>
-    <row r="21" spans="4:4">
-      <c r="D21" s="5"/>
-    </row>
-    <row r="22" spans="4:4">
-      <c r="D22" s="5"/>
-    </row>
-    <row r="23" spans="4:4">
-      <c r="D23" s="5"/>
-    </row>
-    <row r="24" spans="4:4">
-      <c r="D24" s="5"/>
-    </row>
-    <row r="25" spans="4:4">
-      <c r="D25" s="5"/>
-    </row>
-    <row r="26" spans="4:4">
-      <c r="D26" s="5"/>
-    </row>
-    <row r="27" spans="4:4">
-      <c r="D27" s="5"/>
-    </row>
-    <row r="28" spans="4:4">
-      <c r="D28" s="5"/>
-    </row>
-    <row r="29" spans="4:4">
-      <c r="D29" s="5"/>
-    </row>
-    <row r="30" spans="4:4">
-      <c r="D30" s="5"/>
-    </row>
-    <row r="31" spans="4:4">
-      <c r="D31" s="5"/>
-    </row>
-    <row r="32" spans="4:4">
-      <c r="D32" s="5"/>
-    </row>
-    <row r="33" spans="4:4">
-      <c r="D33" s="5"/>
-    </row>
-    <row r="34" spans="4:4">
-      <c r="D34" s="5"/>
-    </row>
-    <row r="35" spans="4:4">
-      <c r="D35" s="5"/>
-    </row>
-    <row r="36" spans="4:4">
-      <c r="D36" s="5"/>
-    </row>
-    <row r="37" spans="4:4">
-      <c r="D37" s="5"/>
-    </row>
-    <row r="38" spans="4:4">
-      <c r="D38" s="5"/>
-    </row>
-    <row r="39" spans="4:4">
-      <c r="D39" s="5"/>
-    </row>
-    <row r="40" spans="4:4">
-      <c r="D40" s="5"/>
-    </row>
-    <row r="41" spans="4:4">
-      <c r="D41" s="5"/>
-    </row>
-    <row r="42" spans="4:4">
-      <c r="D42" s="5"/>
-    </row>
-    <row r="43" spans="4:4">
-      <c r="D43" s="6"/>
-    </row>
-    <row r="44" spans="4:4">
-      <c r="D44" s="6"/>
-    </row>
-    <row r="46" spans="4:4">
-      <c r="D46" s="6"/>
-    </row>
-    <row r="47" spans="4:4">
-      <c r="D47" s="6"/>
-    </row>
-    <row r="48" spans="4:4">
-      <c r="D48" s="8" t="s">
+    </row>
+    <row r="57" spans="4:4">
+      <c r="D57" s="5" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="49" spans="4:4">
-      <c r="D49" s="8" t="s">
+    <row r="58" spans="4:4">
+      <c r="D58" s="3"/>
+    </row>
+    <row r="59" spans="4:4">
+      <c r="D59" s="3"/>
+    </row>
+    <row r="61" spans="4:4">
+      <c r="D61" s="3"/>
+    </row>
+    <row r="62" spans="4:4">
+      <c r="D62" s="3"/>
+    </row>
+    <row r="63" spans="4:4">
+      <c r="D63" s="4" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="50" spans="4:4">
-      <c r="D50" s="8" t="s">
+    <row r="64" spans="4:4">
+      <c r="D64" s="3"/>
+    </row>
+    <row r="65" spans="4:4">
+      <c r="D65" s="6" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="51" spans="4:4">
-      <c r="D51" s="6"/>
-    </row>
-    <row r="52" spans="4:4">
-      <c r="D52" s="6"/>
-    </row>
-    <row r="54" spans="4:4">
-      <c r="D54" s="6"/>
-    </row>
-    <row r="55" spans="4:4">
-      <c r="D55" s="6"/>
-    </row>
-    <row r="56" spans="4:4">
-      <c r="D56" s="7" t="s">
+    <row r="66" spans="4:4">
+      <c r="D66" s="3"/>
+    </row>
+    <row r="67" spans="4:4">
+      <c r="D67" s="5" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="57" spans="4:4">
-      <c r="D57" s="6"/>
-    </row>
-    <row r="58" spans="4:4">
-      <c r="D58" s="9" t="s">
+    <row r="68" spans="4:4">
+      <c r="D68" s="3"/>
+    </row>
+    <row r="69" spans="4:4">
+      <c r="D69" s="7" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="59" spans="4:4">
-      <c r="D59" s="6"/>
-    </row>
-    <row r="60" spans="4:4">
-      <c r="D60" s="8" t="s">
+    <row r="70" spans="4:4">
+      <c r="D70" s="3"/>
+    </row>
+    <row r="71" spans="4:4">
+      <c r="D71" s="5" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="61" spans="4:4">
-      <c r="D61" s="6"/>
-    </row>
-    <row r="62" spans="4:4">
-      <c r="D62" s="10" t="s">
+    <row r="72" spans="4:4">
+      <c r="D72" s="3"/>
+    </row>
+    <row r="73" spans="4:4">
+      <c r="D73" s="8" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="63" spans="4:4">
-      <c r="D63" s="6"/>
-    </row>
-    <row r="64" spans="4:4">
-      <c r="D64" s="8" t="s">
+    <row r="74" spans="4:4">
+      <c r="D74" s="3"/>
+    </row>
+    <row r="75" spans="4:4">
+      <c r="D75" s="3"/>
+    </row>
+    <row r="77" spans="4:4">
+      <c r="D77" s="3"/>
+    </row>
+    <row r="78" spans="4:4">
+      <c r="D78" s="3"/>
+    </row>
+    <row r="79" spans="4:4">
+      <c r="D79" s="4" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="65" spans="4:4">
-      <c r="D65" s="6"/>
-    </row>
-    <row r="66" spans="4:4">
-      <c r="D66" s="11" t="s">
+    <row r="80" spans="4:4">
+      <c r="D80" s="3"/>
+    </row>
+    <row r="81" spans="4:4">
+      <c r="D81" s="6" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="67" spans="4:4">
-      <c r="D67" s="6"/>
-    </row>
-    <row r="68" spans="4:4">
-      <c r="D68" s="6"/>
-    </row>
-    <row r="70" spans="4:4">
-      <c r="D70" s="6"/>
-    </row>
-    <row r="71" spans="4:4">
-      <c r="D71" s="6"/>
-    </row>
-    <row r="72" spans="4:4">
-      <c r="D72" s="7" t="s">
+    <row r="82" spans="4:4">
+      <c r="D82" s="3"/>
+    </row>
+    <row r="83" spans="4:4">
+      <c r="D83" s="9" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="73" spans="4:4">
-      <c r="D73" s="6"/>
-    </row>
-    <row r="74" spans="4:4">
-      <c r="D74" s="9" t="s">
+    <row r="84" spans="4:4">
+      <c r="D84" s="3"/>
+    </row>
+    <row r="85" spans="4:4">
+      <c r="D85" s="7" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="75" spans="4:4">
-      <c r="D75" s="6"/>
-    </row>
-    <row r="76" spans="4:4">
-      <c r="D76" s="12" t="s">
+    <row r="86" spans="4:4">
+      <c r="D86" s="1"/>
+    </row>
+    <row r="87" spans="4:4">
+      <c r="D87" s="10" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="77" spans="4:4">
-      <c r="D77" s="6"/>
-    </row>
-    <row r="78" spans="4:4">
-      <c r="D78" s="10" t="s">
+    <row r="88" spans="4:4">
+      <c r="D88" s="1"/>
+    </row>
+    <row r="89" spans="4:4">
+      <c r="D89" s="11" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="79" spans="4:4">
-      <c r="D79" s="1"/>
-    </row>
-    <row r="80" spans="4:4">
-      <c r="D80" s="13" t="s">
+    <row r="90" spans="4:4">
+      <c r="D90" s="11" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="81" spans="4:4">
-      <c r="D81" s="1"/>
-    </row>
-    <row r="82" spans="4:4">
-      <c r="D82" s="14" t="s">
+    <row r="91" spans="4:4">
+      <c r="D91" s="11"/>
+    </row>
+    <row r="92" spans="4:4">
+      <c r="D92" s="3"/>
+    </row>
+    <row r="93" spans="4:4">
+      <c r="D93" s="3"/>
+    </row>
+    <row r="95" spans="4:4">
+      <c r="D95" s="3"/>
+    </row>
+    <row r="96" spans="4:4">
+      <c r="D96" s="3"/>
+    </row>
+    <row r="97" spans="4:4">
+      <c r="D97" s="9" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="83" spans="4:4">
-      <c r="D83" s="14" t="s">
+    <row r="98" spans="4:4">
+      <c r="D98" s="1"/>
+    </row>
+    <row r="99" spans="4:4">
+      <c r="D99" s="11" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="84" spans="4:4">
-      <c r="D84" s="14"/>
-    </row>
-    <row r="85" spans="4:4">
-      <c r="D85" s="6"/>
-    </row>
-    <row r="86" spans="4:4">
-      <c r="D86" s="6"/>
-    </row>
-    <row r="88" spans="4:4">
-      <c r="D88" s="6"/>
-    </row>
-    <row r="89" spans="4:4">
-      <c r="D89" s="6"/>
-    </row>
-    <row r="90" spans="4:4">
-      <c r="D90" s="12" t="s">
+    <row r="100" spans="4:4">
+      <c r="D100" s="11" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="91" spans="4:4">
-      <c r="D91" s="1"/>
-    </row>
-    <row r="92" spans="4:4">
-      <c r="D92" s="14" t="s">
+    <row r="101" spans="4:4">
+      <c r="D101" s="11"/>
+    </row>
+    <row r="102" spans="4:4">
+      <c r="D102" s="11" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="93" spans="4:4">
-      <c r="D93" s="14" t="s">
+    <row r="103" spans="4:4">
+      <c r="D103" s="12">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="104" spans="4:4">
+      <c r="D104" s="12">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="105" spans="4:4">
+      <c r="D105" s="3"/>
+    </row>
+    <row r="106" spans="4:4">
+      <c r="D106" s="6" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="94" spans="4:4">
-      <c r="D94" s="14"/>
-    </row>
-    <row r="95" spans="4:4">
-      <c r="D95" s="14" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="96" spans="4:4">
-      <c r="D96" s="15">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="97" spans="4:4">
-      <c r="D97" s="15">
-        <v>0.95</v>
-      </c>
-    </row>
-    <row r="98" spans="4:4">
-      <c r="D98" s="6"/>
-    </row>
-    <row r="99" spans="4:4">
-      <c r="D99" s="9" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="100" spans="4:4">
-      <c r="D100" s="6"/>
-    </row>
-    <row r="101" spans="4:4">
-      <c r="D101" s="6"/>
+    <row r="107" spans="4:4">
+      <c r="D107" s="3"/>
+    </row>
+    <row r="108" spans="4:4">
+      <c r="D108" s="3"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D56" r:id="rId1" location="manual-variable-selection" display="http://localhost:8501/ - manual-variable-selection"/>
-    <hyperlink ref="D72" r:id="rId2" location="apply-preprocessing-and-split-dataset" display="http://localhost:8501/ - apply-preprocessing-and-split-dataset"/>
+    <hyperlink ref="D63" r:id="rId1" location="manual-variable-selection" display="http://localhost:8501/ - manual-variable-selection"/>
+    <hyperlink ref="D79" r:id="rId2" location="apply-preprocessing-and-split-dataset" display="http://localhost:8501/ - apply-preprocessing-and-split-dataset"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId3"/>
-  <legacyDrawing r:id="rId4"/>
+  <pageSetup orientation="portrait" r:id="rId3"/>
+  <drawing r:id="rId4"/>
+  <legacyDrawing r:id="rId5"/>
   <controls>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="2050" r:id="rId5" name="Control 2">
-          <controlPr defaultSize="0" r:id="rId6">
+        <control shapeId="2049" r:id="rId6" name="Control 1">
+          <controlPr defaultSize="0" r:id="rId7">
             <anchor moveWithCells="1">
               <from>
                 <xdr:col>3</xdr:col>
                 <xdr:colOff>0</xdr:colOff>
-                <xdr:row>93</xdr:row>
+                <xdr:row>90</xdr:row>
                 <xdr:rowOff>0</xdr:rowOff>
               </from>
               <to>
                 <xdr:col>3</xdr:col>
                 <xdr:colOff>914400</xdr:colOff>
-                <xdr:row>94</xdr:row>
+                <xdr:row>91</xdr:row>
                 <xdr:rowOff>44450</xdr:rowOff>
               </to>
             </anchor>
@@ -1330,24 +1600,24 @@
         </control>
       </mc:Choice>
       <mc:Fallback>
-        <control shapeId="2050" r:id="rId5" name="Control 2"/>
+        <control shapeId="2049" r:id="rId6" name="Control 1"/>
       </mc:Fallback>
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="2049" r:id="rId7" name="Control 1">
-          <controlPr defaultSize="0" r:id="rId6">
+        <control shapeId="2050" r:id="rId8" name="Control 2">
+          <controlPr defaultSize="0" r:id="rId7">
             <anchor moveWithCells="1">
               <from>
                 <xdr:col>3</xdr:col>
                 <xdr:colOff>0</xdr:colOff>
-                <xdr:row>83</xdr:row>
+                <xdr:row>100</xdr:row>
                 <xdr:rowOff>0</xdr:rowOff>
               </from>
               <to>
                 <xdr:col>3</xdr:col>
                 <xdr:colOff>914400</xdr:colOff>
-                <xdr:row>84</xdr:row>
+                <xdr:row>101</xdr:row>
                 <xdr:rowOff>44450</xdr:rowOff>
               </to>
             </anchor>
@@ -1355,7 +1625,7 @@
         </control>
       </mc:Choice>
       <mc:Fallback>
-        <control shapeId="2049" r:id="rId7" name="Control 1"/>
+        <control shapeId="2050" r:id="rId8" name="Control 2"/>
       </mc:Fallback>
     </mc:AlternateContent>
   </controls>

</xml_diff>

<commit_message>
Simplifu the feature selection methods to 5
</commit_message>
<xml_diff>
--- a/Test_Results.xlsx
+++ b/Test_Results.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="52">
   <si>
     <t>Data Selected</t>
   </si>
@@ -311,6 +311,15 @@
   </si>
   <si>
     <t>CGC_3RD_STG_SUCT_PRESS</t>
+  </si>
+  <si>
+    <t>Elastic Net</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Permutation </t>
+  </si>
+  <si>
+    <t>K1301 Turbine HP Steam flow</t>
   </si>
 </sst>
 </file>
@@ -1298,60 +1307,120 @@
       <c r="D29" s="2"/>
     </row>
     <row r="30" spans="1:7">
-      <c r="D30" s="2"/>
+      <c r="B30" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C30" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D30" s="26" t="s">
+        <v>43</v>
+      </c>
+      <c r="E30" s="13">
+        <v>0.67312828741810005</v>
+      </c>
+      <c r="F30" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="G30" s="13" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="31" spans="1:7">
-      <c r="D31" s="2"/>
+      <c r="B31" s="13"/>
+      <c r="C31" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="D31" s="26" t="s">
+        <v>45</v>
+      </c>
+      <c r="E31" s="13">
+        <v>0.89870837811754201</v>
+      </c>
+      <c r="F31" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="G31" s="13"/>
     </row>
     <row r="32" spans="1:7">
-      <c r="D32" s="2"/>
-    </row>
-    <row r="33" spans="4:4">
-      <c r="D33" s="2"/>
-    </row>
-    <row r="34" spans="4:4">
-      <c r="D34" s="2"/>
-    </row>
-    <row r="35" spans="4:4">
-      <c r="D35" s="2"/>
-    </row>
-    <row r="36" spans="4:4">
+      <c r="B32" s="13"/>
+      <c r="C32" s="13"/>
+      <c r="D32" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="E32" s="13"/>
+      <c r="F32" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="G32" s="13"/>
+    </row>
+    <row r="33" spans="2:7">
+      <c r="B33" s="13"/>
+      <c r="C33" s="13"/>
+      <c r="D33" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="E33" s="13"/>
+      <c r="F33" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="G33" s="13"/>
+    </row>
+    <row r="34" spans="2:7">
+      <c r="B34" s="13"/>
+      <c r="C34" s="13"/>
+      <c r="D34" s="13"/>
+      <c r="E34" s="13"/>
+      <c r="F34" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="G34" s="13"/>
+    </row>
+    <row r="35" spans="2:7">
+      <c r="B35" s="13"/>
+      <c r="C35" s="13"/>
+      <c r="D35" s="13"/>
+      <c r="E35" s="13"/>
+      <c r="F35" s="14"/>
+      <c r="G35" s="13"/>
+    </row>
+    <row r="36" spans="2:7">
       <c r="D36" s="2"/>
     </row>
-    <row r="37" spans="4:4">
+    <row r="37" spans="2:7">
       <c r="D37" s="2"/>
     </row>
-    <row r="38" spans="4:4">
+    <row r="38" spans="2:7">
       <c r="D38" s="2"/>
     </row>
-    <row r="39" spans="4:4">
+    <row r="39" spans="2:7">
       <c r="D39" s="2"/>
     </row>
-    <row r="40" spans="4:4">
+    <row r="40" spans="2:7">
       <c r="D40" s="2"/>
     </row>
-    <row r="41" spans="4:4">
+    <row r="41" spans="2:7">
       <c r="D41" s="2"/>
     </row>
-    <row r="42" spans="4:4">
+    <row r="42" spans="2:7">
       <c r="D42" s="2"/>
     </row>
-    <row r="43" spans="4:4">
+    <row r="43" spans="2:7">
       <c r="D43" s="2"/>
     </row>
-    <row r="44" spans="4:4">
+    <row r="44" spans="2:7">
       <c r="D44" s="2"/>
     </row>
-    <row r="45" spans="4:4">
+    <row r="45" spans="2:7">
       <c r="D45" s="2"/>
     </row>
-    <row r="46" spans="4:4">
+    <row r="46" spans="2:7">
       <c r="D46" s="2"/>
     </row>
-    <row r="47" spans="4:4">
+    <row r="47" spans="2:7">
       <c r="D47" s="2"/>
     </row>
-    <row r="48" spans="4:4">
+    <row r="48" spans="2:7">
       <c r="D48" s="2"/>
     </row>
     <row r="49" spans="4:4">
@@ -1580,7 +1649,32 @@
   <controls>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="2049" r:id="rId6" name="Control 1">
+        <control shapeId="2050" r:id="rId6" name="Control 2">
+          <controlPr defaultSize="0" r:id="rId7">
+            <anchor moveWithCells="1">
+              <from>
+                <xdr:col>3</xdr:col>
+                <xdr:colOff>0</xdr:colOff>
+                <xdr:row>100</xdr:row>
+                <xdr:rowOff>0</xdr:rowOff>
+              </from>
+              <to>
+                <xdr:col>3</xdr:col>
+                <xdr:colOff>914400</xdr:colOff>
+                <xdr:row>101</xdr:row>
+                <xdr:rowOff>44450</xdr:rowOff>
+              </to>
+            </anchor>
+          </controlPr>
+        </control>
+      </mc:Choice>
+      <mc:Fallback>
+        <control shapeId="2050" r:id="rId6" name="Control 2"/>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice Requires="x14">
+        <control shapeId="2049" r:id="rId8" name="Control 1">
           <controlPr defaultSize="0" r:id="rId7">
             <anchor moveWithCells="1">
               <from>
@@ -1600,32 +1694,7 @@
         </control>
       </mc:Choice>
       <mc:Fallback>
-        <control shapeId="2049" r:id="rId6" name="Control 1"/>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice Requires="x14">
-        <control shapeId="2050" r:id="rId8" name="Control 2">
-          <controlPr defaultSize="0" r:id="rId7">
-            <anchor moveWithCells="1">
-              <from>
-                <xdr:col>3</xdr:col>
-                <xdr:colOff>0</xdr:colOff>
-                <xdr:row>100</xdr:row>
-                <xdr:rowOff>0</xdr:rowOff>
-              </from>
-              <to>
-                <xdr:col>3</xdr:col>
-                <xdr:colOff>914400</xdr:colOff>
-                <xdr:row>101</xdr:row>
-                <xdr:rowOff>44450</xdr:rowOff>
-              </to>
-            </anchor>
-          </controlPr>
-        </control>
-      </mc:Choice>
-      <mc:Fallback>
-        <control shapeId="2050" r:id="rId8" name="Control 2"/>
+        <control shapeId="2049" r:id="rId8" name="Control 1"/>
       </mc:Fallback>
     </mc:AlternateContent>
   </controls>

</xml_diff>

<commit_message>
Improved the feature selection
</commit_message>
<xml_diff>
--- a/Test_Results.xlsx
+++ b/Test_Results.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="52">
   <si>
     <t>Data Selected</t>
   </si>
@@ -1388,22 +1388,82 @@
       <c r="D36" s="2"/>
     </row>
     <row r="37" spans="2:7">
-      <c r="D37" s="2"/>
+      <c r="B37" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C37" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D37" s="26" t="s">
+        <v>43</v>
+      </c>
+      <c r="E37" s="13">
+        <v>0.67312828741810005</v>
+      </c>
+      <c r="F37" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="G37" s="13" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="38" spans="2:7">
-      <c r="D38" s="2"/>
+      <c r="B38" s="13"/>
+      <c r="C38" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="D38" s="26" t="s">
+        <v>45</v>
+      </c>
+      <c r="E38" s="13">
+        <v>0.89870837811754201</v>
+      </c>
+      <c r="F38" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="G38" s="13"/>
     </row>
     <row r="39" spans="2:7">
-      <c r="D39" s="2"/>
+      <c r="B39" s="13"/>
+      <c r="C39" s="13"/>
+      <c r="D39" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="E39" s="13"/>
+      <c r="F39" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="G39" s="13"/>
     </row>
     <row r="40" spans="2:7">
-      <c r="D40" s="2"/>
+      <c r="B40" s="13"/>
+      <c r="C40" s="13"/>
+      <c r="D40" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="E40" s="13"/>
+      <c r="F40" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="G40" s="13"/>
     </row>
     <row r="41" spans="2:7">
-      <c r="D41" s="2"/>
+      <c r="B41" s="13"/>
+      <c r="C41" s="13"/>
+      <c r="D41" s="13"/>
+      <c r="E41" s="13"/>
+      <c r="F41" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="G41" s="13"/>
     </row>
     <row r="42" spans="2:7">
-      <c r="D42" s="2"/>
+      <c r="B42" s="13"/>
+      <c r="C42" s="13"/>
+      <c r="D42" s="13"/>
+      <c r="E42" s="13"/>
+      <c r="F42" s="14"/>
+      <c r="G42" s="13"/>
     </row>
     <row r="43" spans="2:7">
       <c r="D43" s="2"/>

</xml_diff>

<commit_message>
Updated the feature selection logic
</commit_message>
<xml_diff>
--- a/Test_Results.xlsx
+++ b/Test_Results.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="53">
   <si>
     <t>Data Selected</t>
   </si>
@@ -85,75 +85,6 @@
   </si>
   <si>
     <t>CGC POWER</t>
-  </si>
-  <si>
-    <r>
-      <t>Highly Recommended + Recommended X (2):</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF31333F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8.25"/>
-        <color rgb="FF158237"/>
-        <rFont val="Source Code Pro"/>
-        <family val="3"/>
-      </rPr>
-      <t>CHG_GAS_FLOW_TO_DRYER, DMCTF feed</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Consider X (4):</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF31333F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8.25"/>
-        <color rgb="FF158237"/>
-        <rFont val="Source Code Pro"/>
-        <family val="3"/>
-      </rPr>
-      <t>Average interstage differential pressure, K1301 Turbine HP Steam flow, K1302 5TH STG DISCH PRES, KT1301 TURBINE SPEED (RPM)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Weak Feature (25):</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF31333F"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8.25"/>
-        <color rgb="FF158237"/>
-        <rFont val="Source Code Pro"/>
-        <family val="3"/>
-      </rPr>
-      <t>KT1302 TURBINE SPEED (RPM), Total steam to quench section, Top Reflux Temp, Quench tower overhead temp, Total ET1NE Feed B1206, Total ET1NE Feed B1204, Total ET1NE Feed B1205, Total ET1NE Feed B1209, Total ET1NE Feed B1207, Quench tower feed temp F6_12, K1301_1ST_STG_SUCT_TEMP, Cooling water supply temp, Total ET1NE Feed B1202, Total ET1NE Feed B1203, Total ET1NE Feed B1201, Total ET1NE Feed B1208, Middle Reflux Flow, Total ET1NE Feed B1200, Top Reflux Flow, Quench tower feed temp F1_5, Middle Reflux Temp, B1102 Total ET1NE feed, Avg_MW, B1101 Total ET1NE feed, Overall_COT</t>
-    </r>
   </si>
   <si>
     <t>🎛️ Manual Variable Selection</t>
@@ -320,6 +251,18 @@
   </si>
   <si>
     <t>K1301 Turbine HP Steam flow</t>
+  </si>
+  <si>
+    <t>Lims_R4601_Mi_2</t>
+  </si>
+  <si>
+    <t>case 132 model 132</t>
+  </si>
+  <si>
+    <t>Pump_P4603AB_Hexane_Feed_To_R4601</t>
+  </si>
+  <si>
+    <t>Reactor_R4601_Ethylene_Gas_Analyser_2</t>
   </si>
 </sst>
 </file>
@@ -449,7 +392,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -519,6 +462,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -999,7 +945,7 @@
       <c r="G4" s="16"/>
       <c r="I4" s="16"/>
       <c r="J4" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -1014,7 +960,7 @@
       <c r="G5" s="16"/>
       <c r="I5" s="13"/>
       <c r="J5" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -1100,7 +1046,7 @@
       <c r="B12" s="13"/>
       <c r="C12" s="13"/>
       <c r="D12" s="13" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="E12" s="13"/>
       <c r="F12" s="14" t="s">
@@ -1113,7 +1059,7 @@
       <c r="B13" s="13"/>
       <c r="C13" s="13"/>
       <c r="D13" s="13" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="E13" s="13"/>
       <c r="F13" s="14" t="s">
@@ -1143,7 +1089,7 @@
         <v>18</v>
       </c>
       <c r="D16" s="20" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="E16" s="18">
         <v>-1.05992909334717E-2</v>
@@ -1162,7 +1108,7 @@
         <v>21</v>
       </c>
       <c r="D17" s="20" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="E17" s="18">
         <v>0.75641858263035999</v>
@@ -1230,7 +1176,7 @@
         <v>18</v>
       </c>
       <c r="D23" s="26" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="E23" s="14">
         <v>0.54235839056214397</v>
@@ -1249,7 +1195,7 @@
         <v>21</v>
       </c>
       <c r="D24" s="26" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="E24" s="14">
         <v>0.865024831702778</v>
@@ -1314,7 +1260,7 @@
         <v>18</v>
       </c>
       <c r="D30" s="26" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="E30" s="13">
         <v>0.67312828741810005</v>
@@ -1332,7 +1278,7 @@
         <v>21</v>
       </c>
       <c r="D31" s="26" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="E31" s="13">
         <v>0.89870837811754201</v>
@@ -1346,7 +1292,7 @@
       <c r="B32" s="13"/>
       <c r="C32" s="13"/>
       <c r="D32" s="13" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="E32" s="13"/>
       <c r="F32" s="14" t="s">
@@ -1358,11 +1304,11 @@
       <c r="B33" s="13"/>
       <c r="C33" s="13"/>
       <c r="D33" s="13" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="E33" s="13"/>
       <c r="F33" s="14" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="G33" s="13"/>
     </row>
@@ -1372,7 +1318,7 @@
       <c r="D34" s="13"/>
       <c r="E34" s="13"/>
       <c r="F34" s="14" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="G34" s="13"/>
     </row>
@@ -1395,7 +1341,7 @@
         <v>18</v>
       </c>
       <c r="D37" s="26" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="E37" s="13">
         <v>0.67312828741810005</v>
@@ -1413,7 +1359,7 @@
         <v>21</v>
       </c>
       <c r="D38" s="26" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="E38" s="13">
         <v>0.89870837811754201</v>
@@ -1427,7 +1373,7 @@
       <c r="B39" s="13"/>
       <c r="C39" s="13"/>
       <c r="D39" s="13" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="E39" s="13"/>
       <c r="F39" s="14" t="s">
@@ -1439,11 +1385,11 @@
       <c r="B40" s="13"/>
       <c r="C40" s="13"/>
       <c r="D40" s="13" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="E40" s="13"/>
       <c r="F40" s="14" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="G40" s="13"/>
     </row>
@@ -1453,7 +1399,7 @@
       <c r="D41" s="13"/>
       <c r="E41" s="13"/>
       <c r="F41" s="14" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="G41" s="13"/>
     </row>
@@ -1476,7 +1422,7 @@
         <v>18</v>
       </c>
       <c r="D44" s="26" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="E44" s="13">
         <v>0.75525550494948401</v>
@@ -1494,7 +1440,7 @@
         <v>21</v>
       </c>
       <c r="D45" s="26" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="E45" s="13">
         <v>0.92019836457085802</v>
@@ -1508,7 +1454,7 @@
       <c r="B46" s="13"/>
       <c r="C46" s="13"/>
       <c r="D46" s="13" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="E46" s="13"/>
       <c r="F46" s="14" t="s">
@@ -1522,7 +1468,7 @@
       <c r="D47" s="13"/>
       <c r="E47" s="13"/>
       <c r="F47" s="14" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="G47" s="13"/>
     </row>
@@ -1532,7 +1478,7 @@
       <c r="D48" s="13"/>
       <c r="E48" s="13"/>
       <c r="F48" s="14" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="G48" s="13"/>
     </row>
@@ -1548,28 +1494,59 @@
       <c r="D50" s="3"/>
     </row>
     <row r="51" spans="2:7">
-      <c r="D51" s="3"/>
+      <c r="B51" s="28" t="s">
+        <v>50</v>
+      </c>
+      <c r="C51" s="28" t="s">
+        <v>49</v>
+      </c>
+      <c r="D51" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E51" s="28">
+        <v>0.49469526900315902</v>
+      </c>
+      <c r="F51" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="G51" s="13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="52" spans="2:7">
+      <c r="D52" t="s">
+        <v>51</v>
+      </c>
+      <c r="F52" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="G52" s="13"/>
     </row>
     <row r="53" spans="2:7">
-      <c r="D53" s="3"/>
+      <c r="F53" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="G53" s="13"/>
     </row>
     <row r="54" spans="2:7">
       <c r="D54" s="3"/>
+      <c r="F54" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="G54" s="13"/>
     </row>
     <row r="55" spans="2:7">
-      <c r="D55" s="5" t="s">
-        <v>22</v>
-      </c>
+      <c r="D55" s="5"/>
+      <c r="F55" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="G55" s="13"/>
     </row>
     <row r="56" spans="2:7">
-      <c r="D56" s="5" t="s">
-        <v>23</v>
-      </c>
+      <c r="D56" s="5"/>
     </row>
     <row r="57" spans="2:7">
-      <c r="D57" s="5" t="s">
-        <v>24</v>
-      </c>
+      <c r="D57" s="5"/>
     </row>
     <row r="58" spans="2:7">
       <c r="D58" s="3"/>
@@ -1585,7 +1562,7 @@
     </row>
     <row r="63" spans="2:7">
       <c r="D63" s="4" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="64" spans="2:7">
@@ -1593,7 +1570,7 @@
     </row>
     <row r="65" spans="4:4">
       <c r="D65" s="6" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="66" spans="4:4">
@@ -1601,7 +1578,7 @@
     </row>
     <row r="67" spans="4:4">
       <c r="D67" s="5" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="68" spans="4:4">
@@ -1609,7 +1586,7 @@
     </row>
     <row r="69" spans="4:4">
       <c r="D69" s="7" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="70" spans="4:4">
@@ -1617,7 +1594,7 @@
     </row>
     <row r="71" spans="4:4">
       <c r="D71" s="5" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="72" spans="4:4">
@@ -1625,7 +1602,7 @@
     </row>
     <row r="73" spans="4:4">
       <c r="D73" s="8" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="74" spans="4:4">
@@ -1642,7 +1619,7 @@
     </row>
     <row r="79" spans="4:4">
       <c r="D79" s="4" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="80" spans="4:4">
@@ -1650,7 +1627,7 @@
     </row>
     <row r="81" spans="4:4">
       <c r="D81" s="6" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="82" spans="4:4">
@@ -1658,7 +1635,7 @@
     </row>
     <row r="83" spans="4:4">
       <c r="D83" s="9" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="84" spans="4:4">
@@ -1666,7 +1643,7 @@
     </row>
     <row r="85" spans="4:4">
       <c r="D85" s="7" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="86" spans="4:4">
@@ -1674,7 +1651,7 @@
     </row>
     <row r="87" spans="4:4">
       <c r="D87" s="10" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="88" spans="4:4">
@@ -1682,12 +1659,12 @@
     </row>
     <row r="89" spans="4:4">
       <c r="D89" s="11" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="90" spans="4:4">
       <c r="D90" s="11" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="91" spans="4:4">
@@ -1707,7 +1684,7 @@
     </row>
     <row r="97" spans="4:4">
       <c r="D97" s="9" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="98" spans="4:4">
@@ -1715,12 +1692,12 @@
     </row>
     <row r="99" spans="4:4">
       <c r="D99" s="11" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="100" spans="4:4">
       <c r="D100" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="101" spans="4:4">
@@ -1728,7 +1705,7 @@
     </row>
     <row r="102" spans="4:4">
       <c r="D102" s="11" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="103" spans="4:4">
@@ -1746,7 +1723,7 @@
     </row>
     <row r="106" spans="4:4">
       <c r="D106" s="6" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="107" spans="4:4">

</xml_diff>

<commit_message>
Removed unwanted ui pages
</commit_message>
<xml_diff>
--- a/Test_Results.xlsx
+++ b/Test_Results.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="51">
   <si>
     <t>Data Selected</t>
   </si>
@@ -85,53 +85,6 @@
   </si>
   <si>
     <t>CGC POWER</t>
-  </si>
-  <si>
-    <t>🎛️ Manual Variable Selection</t>
-  </si>
-  <si>
-    <t>Review and adjust the auto-selected X input features and Y target variables.</t>
-  </si>
-  <si>
-    <t>Input Features (X)</t>
-  </si>
-  <si>
-    <t>2 feature(s) auto-selected — check/uncheck to adjust.</t>
-  </si>
-  <si>
-    <t>Target Variables (Y)</t>
-  </si>
-  <si>
-    <r>
-      <t>2</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF94A3B8"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t> X feature(s)  |  </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFF8FAFC"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>2</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF94A3B8"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t> Y target(s)</t>
-    </r>
   </si>
   <si>
     <t>🚀 Apply Preprocessing &amp; Split Dataset</t>
@@ -264,12 +217,35 @@
   <si>
     <t>Reactor_R4601_Ethylene_Gas_Analyser_2</t>
   </si>
+  <si>
+    <t>Cold Data</t>
+  </si>
+  <si>
+    <t>COLD_TRAIN_SEPARATOR_FEED_TEMP</t>
+  </si>
+  <si>
+    <r>
+      <t>Demeth_reboiler_Propylene_flow_ratio</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF31333F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+  </si>
+  <si>
+    <t>Demeth_tower_pressure_control_OP</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="14">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -358,6 +334,18 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF31333F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF31333F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -392,7 +380,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -466,6 +454,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -945,7 +934,7 @@
       <c r="G4" s="16"/>
       <c r="I4" s="16"/>
       <c r="J4" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -960,7 +949,7 @@
       <c r="G5" s="16"/>
       <c r="I5" s="13"/>
       <c r="J5" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -1046,7 +1035,7 @@
       <c r="B12" s="13"/>
       <c r="C12" s="13"/>
       <c r="D12" s="13" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="E12" s="13"/>
       <c r="F12" s="14" t="s">
@@ -1059,7 +1048,7 @@
       <c r="B13" s="13"/>
       <c r="C13" s="13"/>
       <c r="D13" s="13" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="E13" s="13"/>
       <c r="F13" s="14" t="s">
@@ -1089,7 +1078,7 @@
         <v>18</v>
       </c>
       <c r="D16" s="20" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="E16" s="18">
         <v>-1.05992909334717E-2</v>
@@ -1108,7 +1097,7 @@
         <v>21</v>
       </c>
       <c r="D17" s="20" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="E17" s="18">
         <v>0.75641858263035999</v>
@@ -1176,7 +1165,7 @@
         <v>18</v>
       </c>
       <c r="D23" s="26" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="E23" s="14">
         <v>0.54235839056214397</v>
@@ -1195,7 +1184,7 @@
         <v>21</v>
       </c>
       <c r="D24" s="26" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="E24" s="14">
         <v>0.865024831702778</v>
@@ -1260,7 +1249,7 @@
         <v>18</v>
       </c>
       <c r="D30" s="26" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="E30" s="13">
         <v>0.67312828741810005</v>
@@ -1278,7 +1267,7 @@
         <v>21</v>
       </c>
       <c r="D31" s="26" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="E31" s="13">
         <v>0.89870837811754201</v>
@@ -1292,7 +1281,7 @@
       <c r="B32" s="13"/>
       <c r="C32" s="13"/>
       <c r="D32" s="13" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="E32" s="13"/>
       <c r="F32" s="14" t="s">
@@ -1304,11 +1293,11 @@
       <c r="B33" s="13"/>
       <c r="C33" s="13"/>
       <c r="D33" s="13" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="E33" s="13"/>
       <c r="F33" s="14" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="G33" s="13"/>
     </row>
@@ -1318,7 +1307,7 @@
       <c r="D34" s="13"/>
       <c r="E34" s="13"/>
       <c r="F34" s="14" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="G34" s="13"/>
     </row>
@@ -1341,7 +1330,7 @@
         <v>18</v>
       </c>
       <c r="D37" s="26" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="E37" s="13">
         <v>0.67312828741810005</v>
@@ -1359,7 +1348,7 @@
         <v>21</v>
       </c>
       <c r="D38" s="26" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="E38" s="13">
         <v>0.89870837811754201</v>
@@ -1373,7 +1362,7 @@
       <c r="B39" s="13"/>
       <c r="C39" s="13"/>
       <c r="D39" s="13" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="E39" s="13"/>
       <c r="F39" s="14" t="s">
@@ -1385,11 +1374,11 @@
       <c r="B40" s="13"/>
       <c r="C40" s="13"/>
       <c r="D40" s="13" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="E40" s="13"/>
       <c r="F40" s="14" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="G40" s="13"/>
     </row>
@@ -1399,7 +1388,7 @@
       <c r="D41" s="13"/>
       <c r="E41" s="13"/>
       <c r="F41" s="14" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="G41" s="13"/>
     </row>
@@ -1422,7 +1411,7 @@
         <v>18</v>
       </c>
       <c r="D44" s="26" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="E44" s="13">
         <v>0.75525550494948401</v>
@@ -1440,7 +1429,7 @@
         <v>21</v>
       </c>
       <c r="D45" s="26" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="E45" s="13">
         <v>0.92019836457085802</v>
@@ -1454,7 +1443,7 @@
       <c r="B46" s="13"/>
       <c r="C46" s="13"/>
       <c r="D46" s="13" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="E46" s="13"/>
       <c r="F46" s="14" t="s">
@@ -1468,7 +1457,7 @@
       <c r="D47" s="13"/>
       <c r="E47" s="13"/>
       <c r="F47" s="14" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="G47" s="13"/>
     </row>
@@ -1478,7 +1467,7 @@
       <c r="D48" s="13"/>
       <c r="E48" s="13"/>
       <c r="F48" s="14" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="G48" s="13"/>
     </row>
@@ -1495,13 +1484,13 @@
     </row>
     <row r="51" spans="2:7">
       <c r="B51" s="28" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C51" s="28" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="E51" s="28">
         <v>0.49469526900315902</v>
@@ -1515,7 +1504,7 @@
     </row>
     <row r="52" spans="2:7">
       <c r="D52" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="F52" s="14" t="s">
         <v>9</v>
@@ -1531,14 +1520,14 @@
     <row r="54" spans="2:7">
       <c r="D54" s="3"/>
       <c r="F54" s="14" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="G54" s="13"/>
     </row>
     <row r="55" spans="2:7">
       <c r="D55" s="5"/>
       <c r="F55" s="14" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="G55" s="13"/>
     </row>
@@ -1546,10 +1535,23 @@
       <c r="D56" s="5"/>
     </row>
     <row r="57" spans="2:7">
-      <c r="D57" s="5"/>
+      <c r="B57" t="s">
+        <v>47</v>
+      </c>
+      <c r="C57" t="s">
+        <v>48</v>
+      </c>
+      <c r="D57" s="29" t="s">
+        <v>49</v>
+      </c>
+      <c r="E57" s="28">
+        <v>-0.40507977290591402</v>
+      </c>
     </row>
     <row r="58" spans="2:7">
-      <c r="D58" s="3"/>
+      <c r="D58" s="29" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="59" spans="2:7">
       <c r="D59" s="3"/>
@@ -1561,49 +1563,37 @@
       <c r="D62" s="3"/>
     </row>
     <row r="63" spans="2:7">
-      <c r="D63" s="4" t="s">
-        <v>22</v>
-      </c>
+      <c r="D63" s="4"/>
     </row>
     <row r="64" spans="2:7">
       <c r="D64" s="3"/>
     </row>
     <row r="65" spans="4:4">
-      <c r="D65" s="6" t="s">
-        <v>23</v>
-      </c>
+      <c r="D65" s="6"/>
     </row>
     <row r="66" spans="4:4">
       <c r="D66" s="3"/>
     </row>
     <row r="67" spans="4:4">
-      <c r="D67" s="5" t="s">
-        <v>24</v>
-      </c>
+      <c r="D67" s="5"/>
     </row>
     <row r="68" spans="4:4">
       <c r="D68" s="3"/>
     </row>
     <row r="69" spans="4:4">
-      <c r="D69" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="D69" s="7"/>
     </row>
     <row r="70" spans="4:4">
       <c r="D70" s="3"/>
     </row>
     <row r="71" spans="4:4">
-      <c r="D71" s="5" t="s">
-        <v>26</v>
-      </c>
+      <c r="D71" s="5"/>
     </row>
     <row r="72" spans="4:4">
       <c r="D72" s="3"/>
     </row>
     <row r="73" spans="4:4">
-      <c r="D73" s="8" t="s">
-        <v>27</v>
-      </c>
+      <c r="D73" s="8"/>
     </row>
     <row r="74" spans="4:4">
       <c r="D74" s="3"/>
@@ -1619,7 +1609,7 @@
     </row>
     <row r="79" spans="4:4">
       <c r="D79" s="4" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
     </row>
     <row r="80" spans="4:4">
@@ -1627,7 +1617,7 @@
     </row>
     <row r="81" spans="4:4">
       <c r="D81" s="6" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
     </row>
     <row r="82" spans="4:4">
@@ -1635,7 +1625,7 @@
     </row>
     <row r="83" spans="4:4">
       <c r="D83" s="9" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
     </row>
     <row r="84" spans="4:4">
@@ -1643,7 +1633,7 @@
     </row>
     <row r="85" spans="4:4">
       <c r="D85" s="7" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
     </row>
     <row r="86" spans="4:4">
@@ -1651,7 +1641,7 @@
     </row>
     <row r="87" spans="4:4">
       <c r="D87" s="10" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
     </row>
     <row r="88" spans="4:4">
@@ -1659,12 +1649,12 @@
     </row>
     <row r="89" spans="4:4">
       <c r="D89" s="11" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
     </row>
     <row r="90" spans="4:4">
       <c r="D90" s="11" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
     </row>
     <row r="91" spans="4:4">
@@ -1684,7 +1674,7 @@
     </row>
     <row r="97" spans="4:4">
       <c r="D97" s="9" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="98" spans="4:4">
@@ -1692,12 +1682,12 @@
     </row>
     <row r="99" spans="4:4">
       <c r="D99" s="11" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
     </row>
     <row r="100" spans="4:4">
       <c r="D100" s="11" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
     </row>
     <row r="101" spans="4:4">
@@ -1705,7 +1695,7 @@
     </row>
     <row r="102" spans="4:4">
       <c r="D102" s="11" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
     </row>
     <row r="103" spans="4:4">
@@ -1723,7 +1713,7 @@
     </row>
     <row r="106" spans="4:4">
       <c r="D106" s="6" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
     </row>
     <row r="107" spans="4:4">
@@ -1734,18 +1724,42 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D63" r:id="rId1" location="manual-variable-selection" display="http://localhost:8501/ - manual-variable-selection"/>
-    <hyperlink ref="D79" r:id="rId2" location="apply-preprocessing-and-split-dataset" display="http://localhost:8501/ - apply-preprocessing-and-split-dataset"/>
+    <hyperlink ref="D79" r:id="rId1" location="apply-preprocessing-and-split-dataset" display="http://localhost:8501/ - apply-preprocessing-and-split-dataset"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId3"/>
-  <drawing r:id="rId4"/>
-  <legacyDrawing r:id="rId5"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
+  <drawing r:id="rId3"/>
+  <legacyDrawing r:id="rId4"/>
   <controls>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <control shapeId="2049" r:id="rId6" name="Control 1">
-          <controlPr defaultSize="0" r:id="rId7">
+        <control shapeId="2050" r:id="rId5" name="Control 2">
+          <controlPr defaultSize="0" r:id="rId6">
+            <anchor moveWithCells="1">
+              <from>
+                <xdr:col>3</xdr:col>
+                <xdr:colOff>0</xdr:colOff>
+                <xdr:row>100</xdr:row>
+                <xdr:rowOff>0</xdr:rowOff>
+              </from>
+              <to>
+                <xdr:col>3</xdr:col>
+                <xdr:colOff>914400</xdr:colOff>
+                <xdr:row>101</xdr:row>
+                <xdr:rowOff>44450</xdr:rowOff>
+              </to>
+            </anchor>
+          </controlPr>
+        </control>
+      </mc:Choice>
+      <mc:Fallback>
+        <control shapeId="2050" r:id="rId5" name="Control 2"/>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice Requires="x14">
+        <control shapeId="2049" r:id="rId7" name="Control 1">
+          <controlPr defaultSize="0" r:id="rId6">
             <anchor moveWithCells="1">
               <from>
                 <xdr:col>3</xdr:col>
@@ -1764,32 +1778,7 @@
         </control>
       </mc:Choice>
       <mc:Fallback>
-        <control shapeId="2049" r:id="rId6" name="Control 1"/>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice Requires="x14">
-        <control shapeId="2050" r:id="rId8" name="Control 2">
-          <controlPr defaultSize="0" r:id="rId7">
-            <anchor moveWithCells="1">
-              <from>
-                <xdr:col>3</xdr:col>
-                <xdr:colOff>0</xdr:colOff>
-                <xdr:row>100</xdr:row>
-                <xdr:rowOff>0</xdr:rowOff>
-              </from>
-              <to>
-                <xdr:col>3</xdr:col>
-                <xdr:colOff>914400</xdr:colOff>
-                <xdr:row>101</xdr:row>
-                <xdr:rowOff>44450</xdr:rowOff>
-              </to>
-            </anchor>
-          </controlPr>
-        </control>
-      </mc:Choice>
-      <mc:Fallback>
-        <control shapeId="2050" r:id="rId8" name="Control 2"/>
+        <control shapeId="2049" r:id="rId7" name="Control 1"/>
       </mc:Fallback>
     </mc:AlternateContent>
   </controls>

</xml_diff>